<commit_message>
Trocar referencias a fornecedor por 'mapeamento anterior' e apontar badges ao repo publico
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parametro/Leiautes_HCM_Parametro_Extrator_v17.xlsx
+++ b/parametro/Leiautes_HCM_Parametro_Extrator_v17.xlsx
@@ -1164,7 +1164,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fusão de três fontes: leiaute oficial Senior v2.1, mapeamento Fonter e revisão sobre 12.556 XMLs do eSocial.</t>
+          <t>Fusão de três fontes: leiaute oficial Senior v2.1, mapeamento Anterior e revisão sobre 12.556 XMLs do eSocial.</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Mapeamento Fonter?</t>
+          <t>Mapeamento Anterior?</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="L15" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M15" s="30" t="inlineStr">
@@ -3991,7 +3991,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="K15" s="28" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="L15" s="30" t="inlineStr">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="K15" s="28" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="L15" s="30" t="inlineStr">
@@ -5061,7 +5061,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="M15" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N15" s="30" t="inlineStr">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="L16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M16" s="30" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="M15" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N15" s="30" t="inlineStr">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="R16" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S16" s="41" t="n">
@@ -6924,12 +6924,12 @@
       </c>
       <c r="Q17" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R17" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S17" s="41" t="n">
@@ -7005,12 +7005,12 @@
       <c r="P18" s="38" t="n"/>
       <c r="Q18" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S18" s="41" t="n">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="Q16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="R16" s="30" t="inlineStr">
@@ -7512,12 +7512,12 @@
       <c r="T17" s="38" t="n"/>
       <c r="U17" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V17" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W17" s="41" t="n">
@@ -7617,12 +7617,12 @@
       <c r="T18" s="38" t="n"/>
       <c r="U18" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W18" s="41" t="n">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="V19" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="W19" s="41" t="n">
@@ -7822,12 +7822,12 @@
       <c r="T20" s="38" t="n"/>
       <c r="U20" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V20" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W20" s="41" t="n">
@@ -7901,12 +7901,12 @@
       </c>
       <c r="U21" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V21" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W21" s="41" t="n">
@@ -7989,12 +7989,12 @@
       <c r="T22" s="38" t="n"/>
       <c r="U22" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W22" s="41" t="n">
@@ -8093,7 +8093,7 @@
       </c>
       <c r="V23" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="W23" s="41" t="n">
@@ -8192,12 +8192,12 @@
       <c r="T24" s="38" t="n"/>
       <c r="U24" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V24" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W24" s="41" t="n">
@@ -8296,12 +8296,12 @@
       <c r="T25" s="38" t="n"/>
       <c r="U25" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V25" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W25" s="41" t="n">
@@ -8400,12 +8400,12 @@
       <c r="T26" s="38" t="n"/>
       <c r="U26" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V26" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W26" s="41" t="n">
@@ -8492,12 +8492,12 @@
       <c r="T27" s="38" t="n"/>
       <c r="U27" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V27" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W27" s="41" t="n">
@@ -8592,12 +8592,12 @@
       <c r="T28" s="38" t="n"/>
       <c r="U28" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V28" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W28" s="41" t="n">
@@ -8676,7 +8676,7 @@
       </c>
       <c r="V29" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W29" s="47" t="n"/>
@@ -8773,12 +8773,12 @@
       </c>
       <c r="U30" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V30" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="W30" s="55" t="n">
@@ -8791,7 +8791,7 @@
       </c>
       <c r="Y30" s="38" t="inlineStr">
         <is>
-          <t>A tag condIng do Fonter NÃO existe (0 ocorrências em 592 S-2200 + 495 S-2205). A tag correta é trabalhador/trabEstrangeiro/classTrabEstrang. Presente em apenas 1 arquivo (0,2%) - a base praticamente não tem estrangeiros. SUGESTÃO: corrigir a tag e tratar como exceção manual. V11: acrescentado o caminho do trabalhador sem vínculo (S-2300/S-2306). Presença na amostra do piloto: S-2300 0,5%.</t>
+          <t>A tag condIng do Anterior NÃO existe (0 ocorrências em 592 S-2200 + 495 S-2205). A tag correta é trabalhador/trabEstrangeiro/classTrabEstrang. Presente em apenas 1 arquivo (0,2%) - a base praticamente não tem estrangeiros. SUGESTÃO: corrigir a tag e tratar como exceção manual. V11: acrescentado o caminho do trabalhador sem vínculo (S-2300/S-2306). Presença na amostra do piloto: S-2300 0,5%.</t>
         </is>
       </c>
     </row>
@@ -8857,7 +8857,7 @@
       </c>
       <c r="V31" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W31" s="47" t="n"/>
@@ -8930,7 +8930,7 @@
       </c>
       <c r="V32" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W32" s="47" t="n"/>
@@ -9003,7 +9003,7 @@
       </c>
       <c r="V33" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W33" s="47" t="n"/>
@@ -9084,7 +9084,7 @@
       <c r="T34" s="38" t="n"/>
       <c r="U34" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V34" s="40" t="inlineStr">
@@ -9102,7 +9102,7 @@
       </c>
       <c r="Y34" s="38" t="inlineStr">
         <is>
-          <t>CONFIRMADO: documentos/CTPS/nrCtps em 95,9% dos S-2200. Fonter manda vazio - é desperdício. SUGESTÃO: preencher. V11: acrescentado o caminho do trabalhador sem vínculo (S-2300/S-2306). Presença na amostra do piloto: S-2300 52%.</t>
+          <t>CONFIRMADO: documentos/CTPS/nrCtps em 95,9% dos S-2200. Anterior manda vazio - é desperdício. SUGESTÃO: preencher. V11: acrescentado o caminho do trabalhador sem vínculo (S-2300/S-2306). Presença na amostra do piloto: S-2300 52%.</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9176,7 @@
       <c r="T35" s="38" t="n"/>
       <c r="U35" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V35" s="40" t="inlineStr">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="U36" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V36" s="40" t="inlineStr">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="V37" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W37" s="47" t="n"/>
@@ -9450,12 +9450,12 @@
       <c r="T38" s="38" t="n"/>
       <c r="U38" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V38" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W38" s="41" t="n">
@@ -9569,7 +9569,7 @@
       </c>
       <c r="Y39" s="38" t="inlineStr">
         <is>
-          <t>V13: confirmado pelo time que o PIS pode ser extraido. Era 'Enviar vazio' conforme Fonter. trabalhador/nisTrab aparece em 95,9% dos S-2200, 25% dos S-2300 e 2% dos S-2306.</t>
+          <t>V13: confirmado pelo time que o PIS pode ser extraido. Era 'Enviar vazio' conforme Anterior. trabalhador/nisTrab aparece em 95,9% dos S-2200, 25% dos S-2300 e 2% dos S-2306.</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9635,7 @@
       </c>
       <c r="V40" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W40" s="47" t="n"/>
@@ -9711,12 +9711,12 @@
       </c>
       <c r="U41" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V41" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W41" s="41" t="n">
@@ -9799,7 +9799,7 @@
       </c>
       <c r="V42" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W42" s="47" t="n"/>
@@ -9872,7 +9872,7 @@
       </c>
       <c r="V43" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W43" s="47" t="n"/>
@@ -9945,7 +9945,7 @@
       </c>
       <c r="V44" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W44" s="47" t="n"/>
@@ -10018,7 +10018,7 @@
       </c>
       <c r="V45" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W45" s="47" t="n"/>
@@ -10091,7 +10091,7 @@
       </c>
       <c r="V46" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W46" s="47" t="n"/>
@@ -10167,12 +10167,12 @@
       </c>
       <c r="U47" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V47" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W47" s="41" t="n">
@@ -10247,7 +10247,7 @@
       </c>
       <c r="V48" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W48" s="47" t="n"/>
@@ -10327,12 +10327,12 @@
       </c>
       <c r="U49" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V49" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W49" s="55" t="n">
@@ -10418,12 +10418,12 @@
       </c>
       <c r="U50" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V50" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W50" s="55" t="n">
@@ -10526,12 +10526,12 @@
       </c>
       <c r="U51" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V51" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="W51" s="41" t="n">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="Y51" s="38" t="inlineStr">
         <is>
-          <t>CONFIRMADO: os cinco indicadores de deficiência vêm em 100% dos S-2200. SUGESTÃO: DEFFIS = S se qualquer um for S.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Sim", Fonter diz "Não". V11: acrescentado o caminho do trabalhador sem vínculo (S-2300/S-2306). Presença na amostra do piloto: S-2300 100%.</t>
+          <t>CONFIRMADO: os cinco indicadores de deficiência vêm em 100% dos S-2200. SUGESTÃO: DEFFIS = S se qualquer um for S.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Sim", Anterior diz "Não". V11: acrescentado o caminho do trabalhador sem vínculo (S-2300/S-2306). Presença na amostra do piloto: S-2300 100%.</t>
         </is>
       </c>
     </row>
@@ -10630,12 +10630,12 @@
       <c r="T52" s="38" t="n"/>
       <c r="U52" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V52" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W52" s="41" t="n">
@@ -10738,12 +10738,12 @@
       </c>
       <c r="U53" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V53" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="W53" s="41" t="n">
@@ -10843,12 +10843,12 @@
       <c r="T54" s="38" t="n"/>
       <c r="U54" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V54" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W54" s="41" t="n">
@@ -10935,7 +10935,7 @@
       </c>
       <c r="V55" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W55" s="47" t="n"/>
@@ -11028,12 +11028,12 @@
       <c r="T56" s="38" t="n"/>
       <c r="U56" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="V56" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W56" s="41" t="n">
@@ -11120,7 +11120,7 @@
       </c>
       <c r="V57" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W57" s="47" t="n"/>
@@ -11201,7 +11201,7 @@
       </c>
       <c r="V58" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W58" s="47" t="n"/>
@@ -11282,7 +11282,7 @@
       </c>
       <c r="V59" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W59" s="47" t="n"/>
@@ -11455,7 +11455,7 @@
       </c>
       <c r="V61" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W61" s="47" t="n"/>
@@ -11536,7 +11536,7 @@
       </c>
       <c r="V62" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W62" s="47" t="n"/>
@@ -11617,7 +11617,7 @@
       </c>
       <c r="V63" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W63" s="47" t="n"/>
@@ -11698,7 +11698,7 @@
       </c>
       <c r="V64" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W64" s="47" t="n"/>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="V65" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W65" s="47" t="n"/>
@@ -11860,7 +11860,7 @@
       </c>
       <c r="V66" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W66" s="47" t="n"/>
@@ -11944,7 +11944,7 @@
       <c r="T67" s="38" t="n"/>
       <c r="U67" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V67" s="40" t="inlineStr">
@@ -12027,12 +12027,12 @@
       <c r="T68" s="38" t="n"/>
       <c r="U68" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="V68" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W68" s="41" t="n">
@@ -12107,7 +12107,7 @@
       </c>
       <c r="V69" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="W69" s="47" t="n"/>
@@ -12290,7 +12290,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -12360,7 +12360,7 @@
       </c>
       <c r="M16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N16" s="30" t="inlineStr">
@@ -12471,12 +12471,12 @@
       <c r="P17" s="38" t="n"/>
       <c r="Q17" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R17" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S17" s="41" t="n">
@@ -12564,12 +12564,12 @@
       <c r="P18" s="38" t="n"/>
       <c r="Q18" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S18" s="41" t="n">
@@ -12653,12 +12653,12 @@
       <c r="P19" s="38" t="n"/>
       <c r="Q19" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R19" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S19" s="41" t="n">
@@ -12836,7 +12836,7 @@
       </c>
       <c r="R21" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S21" s="41" t="n">
@@ -12924,12 +12924,12 @@
       <c r="P22" s="38" t="n"/>
       <c r="Q22" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S22" s="41" t="n">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="R23" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S23" s="41" t="n">
@@ -13102,12 +13102,12 @@
       <c r="P24" s="38" t="n"/>
       <c r="Q24" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R24" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S24" s="41" t="n">
@@ -13183,12 +13183,12 @@
       <c r="P25" s="38" t="n"/>
       <c r="Q25" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R25" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S25" s="41" t="n">
@@ -13276,12 +13276,12 @@
       <c r="P26" s="38" t="n"/>
       <c r="Q26" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R26" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S26" s="41" t="n">
@@ -13357,12 +13357,12 @@
       <c r="P27" s="38" t="n"/>
       <c r="Q27" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R27" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S27" s="41" t="n">
@@ -13438,12 +13438,12 @@
       <c r="P28" s="38" t="n"/>
       <c r="Q28" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R28" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S28" s="41" t="n">
@@ -13519,12 +13519,12 @@
       <c r="P29" s="38" t="n"/>
       <c r="Q29" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R29" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S29" s="49" t="n">
@@ -13613,7 +13613,7 @@
       </c>
       <c r="R30" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S30" s="41" t="n">
@@ -13697,7 +13697,7 @@
       </c>
       <c r="Q31" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R31" s="40" t="inlineStr">
@@ -13715,7 +13715,7 @@
       </c>
       <c r="U31" s="38" t="inlineStr">
         <is>
-          <t>CORREÇÃO: existe - nascimento/uf no S-2205 (64%) e no S-2200 (2,2%). SUGESTÃO: usar a tag direta e derivar do codMunic só onde faltar.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Fonter diz "Sim".</t>
+          <t>CORREÇÃO: existe - nascimento/uf no S-2205 (64%) e no S-2200 (2,2%). SUGESTÃO: usar a tag direta e derivar do codMunic só onde faltar.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Anterior diz "Sim".</t>
         </is>
       </c>
     </row>
@@ -13786,7 +13786,7 @@
       </c>
       <c r="Q32" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R32" s="40" t="inlineStr">
@@ -13804,7 +13804,7 @@
       </c>
       <c r="U32" s="38" t="inlineStr">
         <is>
-          <t>Confirmado: nascimento/codMunic em 95,3% dos S-2200. SUGESTÃO: usar o XML em vez de relatório.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Fonter diz "Sim".</t>
+          <t>Confirmado: nascimento/codMunic em 95,3% dos S-2200. SUGESTÃO: usar o XML em vez de relatório.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Anterior diz "Sim".</t>
         </is>
       </c>
     </row>
@@ -13875,7 +13875,7 @@
       </c>
       <c r="Q33" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R33" s="40" t="inlineStr">
@@ -13964,7 +13964,7 @@
       </c>
       <c r="Q34" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R34" s="40" t="inlineStr">
@@ -14046,7 +14046,7 @@
       </c>
       <c r="R35" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S35" s="47" t="n"/>
@@ -14125,7 +14125,7 @@
       </c>
       <c r="R36" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S36" s="47" t="n"/>
@@ -14281,7 +14281,7 @@
       </c>
       <c r="R38" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S38" s="47" t="n"/>
@@ -14352,7 +14352,7 @@
       </c>
       <c r="R39" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S39" s="47" t="n"/>
@@ -14423,7 +14423,7 @@
       </c>
       <c r="R40" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S40" s="47" t="n"/>
@@ -14749,7 +14749,7 @@
       </c>
       <c r="R44" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S44" s="47" t="n"/>
@@ -14913,7 +14913,7 @@
       </c>
       <c r="R46" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S46" s="47" t="n"/>
@@ -14984,7 +14984,7 @@
       </c>
       <c r="R47" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S47" s="47" t="n"/>
@@ -15140,7 +15140,7 @@
       </c>
       <c r="R49" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S49" s="47" t="n"/>
@@ -15211,7 +15211,7 @@
       </c>
       <c r="R50" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S50" s="47" t="n"/>
@@ -15374,7 +15374,7 @@
       </c>
       <c r="Q52" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R52" s="40" t="inlineStr">
@@ -15456,7 +15456,7 @@
       </c>
       <c r="R53" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S53" s="47" t="n"/>
@@ -15539,7 +15539,7 @@
       </c>
       <c r="R54" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S54" s="55" t="n">
@@ -15552,7 +15552,7 @@
       </c>
       <c r="U54" s="38" t="inlineStr">
         <is>
-          <t>contato/emailPrinc existe, mas em apenas 2,5% dos S-2200. O mapeamento Fonter está certo; só não espere volume. SUGESTÃO: manter e avisar o cliente que o e-mail virá quase todo vazio.</t>
+          <t>contato/emailPrinc existe, mas em apenas 2,5% dos S-2200. O mapeamento Anterior está certo; só não espere volume. SUGESTÃO: manter e avisar o cliente que o e-mail virá quase todo vazio.</t>
         </is>
       </c>
     </row>
@@ -15616,7 +15616,7 @@
       </c>
       <c r="R55" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S55" s="47" t="n"/>
@@ -15690,7 +15690,7 @@
       <c r="P56" s="38" t="n"/>
       <c r="Q56" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R56" s="40" t="inlineStr">
@@ -15772,7 +15772,7 @@
       </c>
       <c r="R57" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S57" s="47" t="n"/>
@@ -15859,7 +15859,7 @@
       </c>
       <c r="R58" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S58" s="55" t="n">
@@ -15948,7 +15948,7 @@
       </c>
       <c r="R59" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S59" s="55" t="n">
@@ -16025,7 +16025,7 @@
       </c>
       <c r="R60" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S60" s="47" t="n"/>
@@ -16096,7 +16096,7 @@
       </c>
       <c r="R61" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S61" s="47" t="n"/>
@@ -16250,7 +16250,7 @@
       </c>
       <c r="P63" s="38" t="inlineStr">
         <is>
-          <t>nmSoc confirmado: 0,5% dos S-2200 e 4,6% dos S-2205. Mapeamento Fonter correto, volume baixo.</t>
+          <t>nmSoc confirmado: 0,5% dos S-2200 e 4,6% dos S-2205. Mapeamento Anterior correto, volume baixo.</t>
         </is>
       </c>
       <c r="Q63" s="38" t="inlineStr">
@@ -16260,7 +16260,7 @@
       </c>
       <c r="R63" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S63" s="55" t="n">
@@ -16273,7 +16273,7 @@
       </c>
       <c r="U63" s="38" t="inlineStr">
         <is>
-          <t>nmSoc confirmado: 0,5% dos S-2200 e 4,6% dos S-2205. Mapeamento Fonter correto, volume baixo.</t>
+          <t>nmSoc confirmado: 0,5% dos S-2200 e 4,6% dos S-2205. Mapeamento Anterior correto, volume baixo.</t>
         </is>
       </c>
     </row>
@@ -16449,7 +16449,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -16519,7 +16519,7 @@
       </c>
       <c r="M16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N16" s="30" t="inlineStr">
@@ -16628,12 +16628,12 @@
       <c r="P17" s="38" t="n"/>
       <c r="Q17" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R17" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S17" s="41" t="n">
@@ -16730,7 +16730,7 @@
       </c>
       <c r="R18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S18" s="55" t="n">
@@ -16816,12 +16816,12 @@
       <c r="P19" s="38" t="n"/>
       <c r="Q19" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R19" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S19" s="41" t="n">
@@ -16900,17 +16900,17 @@
       </c>
       <c r="P20" s="38" t="inlineStr">
         <is>
-          <t>Na linha gerada a partir do S-2299 usar infoDeslig/dtDeslig (o Fonter escreveu datDeslig).</t>
+          <t>Na linha gerada a partir do S-2299 usar infoDeslig/dtDeslig (o Anterior escreveu datDeslig).</t>
         </is>
       </c>
       <c r="Q20" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R20" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S20" s="49" t="n">
@@ -16987,7 +16987,7 @@
       </c>
       <c r="R21" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S21" s="47" t="n"/>
@@ -17057,12 +17057,12 @@
       <c r="P22" s="38" t="n"/>
       <c r="Q22" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S22" s="49" t="n">
@@ -17135,7 +17135,7 @@
       </c>
       <c r="R23" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S23" s="47" t="n"/>
@@ -17206,7 +17206,7 @@
       </c>
       <c r="R24" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S24" s="47" t="n"/>
@@ -17301,7 +17301,7 @@
       </c>
       <c r="R25" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S25" s="49" t="n">
@@ -17393,12 +17393,12 @@
       <c r="P26" s="38" t="n"/>
       <c r="Q26" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R26" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S26" s="41" t="n">
@@ -17563,12 +17563,12 @@
       <c r="P28" s="38" t="n"/>
       <c r="Q28" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R28" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S28" s="55" t="n">
@@ -17662,7 +17662,7 @@
       </c>
       <c r="U29" s="38" t="inlineStr">
         <is>
-          <t>CORREÇÃO: existe - infoAtestado/codCID em 12,1% dos S-2230. Fonter manda vazio. SUGESTÃO: preencher os afastamentos com atestado.</t>
+          <t>CORREÇÃO: existe - infoAtestado/codCID em 12,1% dos S-2230. Anterior manda vazio. SUGESTÃO: preencher os afastamentos com atestado.</t>
         </is>
       </c>
     </row>
@@ -18074,7 +18074,7 @@
       </c>
       <c r="R34" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S34" s="47" t="n"/>
@@ -18273,7 +18273,7 @@
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -18355,7 +18355,7 @@
       </c>
       <c r="M19" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N19" s="30" t="inlineStr">
@@ -18470,12 +18470,12 @@
       <c r="P20" s="38" t="n"/>
       <c r="Q20" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R20" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S20" s="41" t="n">
@@ -18567,12 +18567,12 @@
       <c r="P21" s="38" t="n"/>
       <c r="Q21" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R21" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S21" s="41" t="n">
@@ -18656,12 +18656,12 @@
       <c r="P22" s="38" t="n"/>
       <c r="Q22" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S22" s="41" t="n">
@@ -18741,12 +18741,12 @@
       </c>
       <c r="Q23" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R23" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S23" s="49" t="n">
@@ -18822,12 +18822,12 @@
       </c>
       <c r="Q24" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R24" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S24" s="47" t="n"/>
@@ -18918,7 +18918,7 @@
       </c>
       <c r="R25" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S25" s="60" t="n">
@@ -18999,7 +18999,7 @@
       </c>
       <c r="R26" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S26" s="47" t="n"/>
@@ -19077,7 +19077,7 @@
     <row r="1" ht="18" customHeight="1" s="104">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>◆ Validação da amostra - 2ª rodada (revisão sobre os XMLs, não faz parte do Fonter original)</t>
+          <t>◆ Validação da amostra - 2ª rodada (revisão sobre os XMLs, não faz parte do Anterior original)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -19921,7 +19921,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -19981,7 +19981,7 @@
       </c>
       <c r="K17" s="28" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="L17" s="30" t="inlineStr">
@@ -20591,7 +20591,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -20673,7 +20673,7 @@
       </c>
       <c r="M18" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N18" s="30" t="inlineStr">
@@ -21248,7 +21248,7 @@
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -21325,7 +21325,7 @@
       </c>
       <c r="L19" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M19" s="30" t="inlineStr">
@@ -22034,7 +22034,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -22099,7 +22099,7 @@
       </c>
       <c r="L16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M16" s="30" t="inlineStr">
@@ -22209,12 +22209,12 @@
       <c r="O17" s="38" t="n"/>
       <c r="P17" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="Q17" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R17" s="41" t="n">
@@ -22301,12 +22301,12 @@
       <c r="O18" s="38" t="n"/>
       <c r="P18" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="Q18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R18" s="41" t="n">
@@ -22385,12 +22385,12 @@
       <c r="O19" s="38" t="n"/>
       <c r="P19" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="Q19" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R19" s="41" t="n">
@@ -22465,12 +22465,12 @@
       </c>
       <c r="P20" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="Q20" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="R20" s="41" t="n">
@@ -22562,7 +22562,7 @@
       </c>
       <c r="Q21" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="R21" s="41" t="n">
@@ -22759,7 +22759,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -22836,7 +22836,7 @@
       </c>
       <c r="L18" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M18" s="30" t="inlineStr">
@@ -23578,7 +23578,7 @@
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -23648,7 +23648,7 @@
       </c>
       <c r="M18" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N18" s="30" t="inlineStr">
@@ -23759,12 +23759,12 @@
       <c r="P19" s="38" t="n"/>
       <c r="Q19" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R19" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S19" s="41" t="n">
@@ -23852,12 +23852,12 @@
       <c r="P20" s="38" t="n"/>
       <c r="Q20" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R20" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S20" s="41" t="n">
@@ -23937,12 +23937,12 @@
       <c r="P21" s="38" t="n"/>
       <c r="Q21" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R21" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S21" s="41" t="n">
@@ -24014,12 +24014,12 @@
       <c r="P22" s="38" t="n"/>
       <c r="Q22" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S22" s="41" t="n">
@@ -24104,7 +24104,7 @@
       </c>
       <c r="R23" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S23" s="41" t="n">
@@ -24201,7 +24201,7 @@
       </c>
       <c r="R24" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S24" s="41" t="n">
@@ -24298,7 +24298,7 @@
       </c>
       <c r="R25" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S25" s="41" t="n">
@@ -24478,7 +24478,7 @@
       </c>
       <c r="P27" s="38" t="inlineStr">
         <is>
-          <t>unificar a regra de FICREG entre 1013 e 1021.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Fonter diz "Sim".</t>
+          <t>unificar a regra de FICREG entre 1013 e 1021.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Anterior diz "Sim".</t>
         </is>
       </c>
       <c r="Q27" s="38" t="inlineStr">
@@ -24488,7 +24488,7 @@
       </c>
       <c r="R27" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S27" s="41" t="n">
@@ -24576,12 +24576,12 @@
       <c r="P28" s="38" t="n"/>
       <c r="Q28" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R28" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S28" s="41" t="n">
@@ -24765,7 +24765,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -24825,7 +24825,7 @@
       </c>
       <c r="K16" s="28" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="L16" s="30" t="inlineStr">
@@ -25422,7 +25422,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -25482,7 +25482,7 @@
       </c>
       <c r="K15" s="28" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="L15" s="30" t="inlineStr">
@@ -25842,7 +25842,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -25902,7 +25902,7 @@
       </c>
       <c r="K17" s="28" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="L17" s="30" t="inlineStr">
@@ -26437,7 +26437,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -26507,7 +26507,7 @@
       </c>
       <c r="M16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N16" s="30" t="inlineStr">
@@ -27237,17 +27237,17 @@
       </c>
       <c r="C4" s="88" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="D4" s="89" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="E4" s="90" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="F4" s="91" t="inlineStr">
@@ -28489,7 +28489,7 @@
     <row r="55" ht="15.6" customHeight="1" s="104">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>Campos onde a revisão substituiu o mapeamento Fonter</t>
+          <t>Campos onde a revisão substituiu o mapeamento Anterior</t>
         </is>
       </c>
     </row>
@@ -29247,7 +29247,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -29329,7 +29329,7 @@
       </c>
       <c r="M17" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N17" s="30" t="inlineStr">
@@ -29440,12 +29440,12 @@
       <c r="P18" s="38" t="n"/>
       <c r="Q18" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S18" s="41" t="n">
@@ -29533,12 +29533,12 @@
       <c r="P19" s="38" t="n"/>
       <c r="Q19" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R19" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S19" s="41" t="n">
@@ -29622,12 +29622,12 @@
       <c r="P20" s="38" t="n"/>
       <c r="Q20" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R20" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S20" s="41" t="n">
@@ -29711,12 +29711,12 @@
       </c>
       <c r="Q21" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R21" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S21" s="41" t="n">
@@ -29804,12 +29804,12 @@
       <c r="P22" s="38" t="n"/>
       <c r="Q22" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S22" s="41" t="n">
@@ -29998,7 +29998,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -30080,7 +30080,7 @@
       </c>
       <c r="M17" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N17" s="30" t="inlineStr">
@@ -30191,12 +30191,12 @@
       <c r="P18" s="38" t="n"/>
       <c r="Q18" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S18" s="41" t="n">
@@ -30284,12 +30284,12 @@
       <c r="P19" s="38" t="n"/>
       <c r="Q19" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R19" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S19" s="41" t="n">
@@ -30386,7 +30386,7 @@
       </c>
       <c r="R20" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S20" s="41" t="n">
@@ -30470,12 +30470,12 @@
       </c>
       <c r="Q21" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R21" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S21" s="41" t="n">
@@ -30563,12 +30563,12 @@
       <c r="P22" s="38" t="n"/>
       <c r="Q22" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S22" s="41" t="n">
@@ -30765,7 +30765,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -30842,7 +30842,7 @@
       </c>
       <c r="L18" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M18" s="30" t="inlineStr">
@@ -31544,7 +31544,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -31626,7 +31626,7 @@
       </c>
       <c r="M17" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N17" s="30" t="inlineStr">
@@ -31741,12 +31741,12 @@
       <c r="P18" s="38" t="n"/>
       <c r="Q18" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S18" s="41" t="n">
@@ -31838,12 +31838,12 @@
       <c r="P19" s="38" t="n"/>
       <c r="Q19" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R19" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S19" s="41" t="n">
@@ -31940,7 +31940,7 @@
       </c>
       <c r="R20" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S20" s="41" t="n">
@@ -32024,12 +32024,12 @@
       </c>
       <c r="Q21" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R21" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S21" s="49" t="n">
@@ -32101,12 +32101,12 @@
       </c>
       <c r="Q22" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S22" s="47" t="n"/>
@@ -32181,7 +32181,7 @@
       </c>
       <c r="R23" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S23" s="47" t="n"/>
@@ -32259,12 +32259,12 @@
       <c r="P24" s="38" t="n"/>
       <c r="Q24" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R24" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S24" s="41" t="n">
@@ -32361,7 +32361,7 @@
       </c>
       <c r="R25" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S25" s="41" t="n">
@@ -32445,7 +32445,7 @@
       </c>
       <c r="Q26" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R26" s="40" t="inlineStr">
@@ -32646,7 +32646,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -32735,7 +32735,7 @@
       </c>
       <c r="N16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="O16" s="30" t="inlineStr">
@@ -32851,12 +32851,12 @@
       <c r="Q17" s="38" t="n"/>
       <c r="R17" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="S17" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T17" s="41" t="n">
@@ -32949,12 +32949,12 @@
       <c r="Q18" s="38" t="n"/>
       <c r="R18" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="S18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T18" s="41" t="n">
@@ -33048,7 +33048,7 @@
       </c>
       <c r="S19" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="T19" s="41" t="n">
@@ -33121,12 +33121,12 @@
       </c>
       <c r="R20" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="S20" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T20" s="47" t="n"/>
@@ -33201,12 +33201,12 @@
       <c r="Q21" s="38" t="n"/>
       <c r="R21" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="S21" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T21" s="49" t="n">
@@ -33280,7 +33280,7 @@
       </c>
       <c r="S22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T22" s="47" t="n"/>
@@ -33367,12 +33367,12 @@
       <c r="Q23" s="38" t="n"/>
       <c r="R23" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="S23" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T23" s="49" t="n">
@@ -33523,12 +33523,12 @@
       <c r="Q25" s="38" t="n"/>
       <c r="R25" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="S25" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T25" s="49" t="n">
@@ -33601,12 +33601,12 @@
       <c r="Q26" s="38" t="n"/>
       <c r="R26" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="S26" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T26" s="41" t="n">
@@ -33691,7 +33691,7 @@
       </c>
       <c r="R27" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="S27" s="40" t="inlineStr">
@@ -33774,7 +33774,7 @@
       </c>
       <c r="S28" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T28" s="47" t="n"/>
@@ -33846,7 +33846,7 @@
       </c>
       <c r="S29" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T29" s="47" t="n"/>
@@ -33918,7 +33918,7 @@
       </c>
       <c r="S30" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T30" s="47" t="n"/>
@@ -33990,7 +33990,7 @@
       </c>
       <c r="S31" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T31" s="47" t="n"/>
@@ -34061,12 +34061,12 @@
       <c r="Q32" s="38" t="n"/>
       <c r="R32" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="S32" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T32" s="49" t="n">
@@ -34147,12 +34147,12 @@
       </c>
       <c r="R33" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="S33" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T33" s="41" t="n">
@@ -34230,7 +34230,7 @@
       </c>
       <c r="S34" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T34" s="47" t="n"/>
@@ -34302,7 +34302,7 @@
       </c>
       <c r="S35" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T35" s="47" t="n"/>
@@ -34377,7 +34377,7 @@
       <c r="Q36" s="38" t="n"/>
       <c r="R36" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="S36" s="40" t="inlineStr">
@@ -34460,7 +34460,7 @@
       </c>
       <c r="S37" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T37" s="47" t="n"/>
@@ -34532,7 +34532,7 @@
       </c>
       <c r="S38" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T38" s="47" t="n"/>
@@ -34604,7 +34604,7 @@
       </c>
       <c r="S39" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T39" s="47" t="n"/>
@@ -34676,7 +34676,7 @@
       </c>
       <c r="S40" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T40" s="47" t="n"/>
@@ -34756,7 +34756,7 @@
       </c>
       <c r="S41" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T41" s="47" t="n"/>
@@ -34832,7 +34832,7 @@
       </c>
       <c r="S42" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T42" s="47" t="n"/>
@@ -34919,12 +34919,12 @@
       <c r="Q43" s="38" t="n"/>
       <c r="R43" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="S43" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T43" s="49" t="n">
@@ -35001,12 +35001,12 @@
       <c r="Q44" s="38" t="n"/>
       <c r="R44" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="S44" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T44" s="49" t="n">
@@ -35080,7 +35080,7 @@
       </c>
       <c r="S45" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T45" s="47" t="n"/>
@@ -35152,7 +35152,7 @@
       </c>
       <c r="S46" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T46" s="47" t="n"/>
@@ -35224,7 +35224,7 @@
       </c>
       <c r="S47" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T47" s="47" t="n"/>
@@ -35296,7 +35296,7 @@
       </c>
       <c r="S48" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T48" s="47" t="n"/>
@@ -35368,7 +35368,7 @@
       </c>
       <c r="S49" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T49" s="47" t="n"/>
@@ -35440,7 +35440,7 @@
       </c>
       <c r="S50" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T50" s="47" t="n"/>
@@ -35512,7 +35512,7 @@
       </c>
       <c r="S51" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T51" s="47" t="n"/>
@@ -35592,7 +35592,7 @@
       </c>
       <c r="S52" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T52" s="47" t="n"/>
@@ -35664,7 +35664,7 @@
       </c>
       <c r="S53" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T53" s="47" t="n"/>
@@ -35736,7 +35736,7 @@
       </c>
       <c r="S54" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T54" s="47" t="n"/>
@@ -35808,7 +35808,7 @@
       </c>
       <c r="S55" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="T55" s="47" t="n"/>
@@ -35991,7 +35991,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -36061,7 +36061,7 @@
       </c>
       <c r="M16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N16" s="30" t="inlineStr">
@@ -37386,7 +37386,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -37470,7 +37470,7 @@
       </c>
       <c r="N17" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="O17" s="30" t="inlineStr">
@@ -38603,7 +38603,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -38682,7 +38682,7 @@
       </c>
       <c r="M17" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N17" s="30" t="inlineStr">
@@ -39659,7 +39659,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -39719,7 +39719,7 @@
       </c>
       <c r="K17" s="28" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="L17" s="30" t="inlineStr">
@@ -40518,7 +40518,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -40619,7 +40619,7 @@
       </c>
       <c r="O17" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="P17" s="30" t="inlineStr">
@@ -42705,7 +42705,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -42770,7 +42770,7 @@
       </c>
       <c r="L17" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M17" s="30" t="inlineStr">
@@ -43501,7 +43501,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -43580,7 +43580,7 @@
       </c>
       <c r="M16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N16" s="30" t="inlineStr">
@@ -45074,7 +45074,7 @@
       </c>
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fronter_Leiautes eSocial_1038.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Fronter_Leiautes eSocial_1038.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -45165,7 +45165,7 @@
       </c>
       <c r="M20" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N20" s="30" t="inlineStr">
@@ -45272,12 +45272,12 @@
       <c r="P21" s="38" t="n"/>
       <c r="Q21" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R21" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S21" s="41" t="n">
@@ -45455,7 +45455,7 @@
       </c>
       <c r="R23" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S23" s="41" t="n">
@@ -45544,7 +45544,7 @@
       </c>
       <c r="R24" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S24" s="41" t="n">
@@ -45710,7 +45710,7 @@
       </c>
       <c r="R26" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S26" s="41" t="n">
@@ -45790,12 +45790,12 @@
       </c>
       <c r="Q27" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R27" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S27" s="41" t="n">
@@ -45808,7 +45808,7 @@
       </c>
       <c r="U27" s="38" t="inlineStr">
         <is>
-          <t>CONFIRMADO: dos 13.812 itens de verba, 3.781 têm qtdRubr e 4.989 têm fatorRubr - ou seja, mais da metade não tem qtdRubr. SUGESTÃO: REFEVE = qtdRubr, senão fatorRubr, senão vazio.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Fonter diz "Sim".</t>
+          <t>CONFIRMADO: dos 13.812 itens de verba, 3.781 têm qtdRubr e 4.989 têm fatorRubr - ou seja, mais da metade não tem qtdRubr. SUGESTÃO: REFEVE = qtdRubr, senão fatorRubr, senão vazio.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Anterior diz "Sim".</t>
         </is>
       </c>
     </row>
@@ -45871,12 +45871,12 @@
       <c r="P28" s="38" t="n"/>
       <c r="Q28" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R28" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S28" s="41" t="n">
@@ -46077,7 +46077,7 @@
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -46156,7 +46156,7 @@
       </c>
       <c r="M18" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N18" s="30" t="inlineStr">
@@ -47200,7 +47200,7 @@
       </c>
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fronter_Leiautes eSocial 1040.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Fronter_Leiautes eSocial 1040.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -47279,7 +47279,7 @@
       </c>
       <c r="M19" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N19" s="30" t="inlineStr">
@@ -47386,12 +47386,12 @@
       <c r="P20" s="38" t="n"/>
       <c r="Q20" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R20" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S20" s="41" t="n">
@@ -47475,12 +47475,12 @@
       <c r="P21" s="38" t="n"/>
       <c r="Q21" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R21" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S21" s="41" t="n">
@@ -47565,7 +47565,7 @@
       </c>
       <c r="R22" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S22" s="41" t="n">
@@ -47816,7 +47816,7 @@
       </c>
       <c r="R25" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S25" s="41" t="n">
@@ -47896,12 +47896,12 @@
       </c>
       <c r="Q26" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R26" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S26" s="41" t="n">
@@ -47914,7 +47914,7 @@
       </c>
       <c r="U26" s="38" t="inlineStr">
         <is>
-          <t>CONFIRMADO: dos 10.799 itens do S-1200, apenas 855 têm qtdRubr e 2.598 têm fatorRubr. SUGESTÃO: REFEVE = qtdRubr, senão fatorRubr, senão vazio - senão 85% das linhas ficam sem referência.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Fonter diz "Sim".</t>
+          <t>CONFIRMADO: dos 10.799 itens do S-1200, apenas 855 têm qtdRubr e 2.598 têm fatorRubr. SUGESTÃO: REFEVE = qtdRubr, senão fatorRubr, senão vazio - senão 85% das linhas ficam sem referência.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Anterior diz "Sim".</t>
         </is>
       </c>
     </row>
@@ -47977,12 +47977,12 @@
       <c r="P27" s="38" t="n"/>
       <c r="Q27" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R27" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S27" s="41" t="n">
@@ -48088,7 +48088,7 @@
       </c>
       <c r="U28" s="38" t="inlineStr">
         <is>
-          <t>CONFIRMADO: ideEvento/indApuracao em 100% dos S-1200. SUGESTÃO: 1 -&gt; cálculo 11 (mensal), 2 -&gt; cálculo 32 (13º).  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Fonter diz "Sim".</t>
+          <t>CONFIRMADO: ideEvento/indApuracao em 100% dos S-1200. SUGESTÃO: 1 -&gt; cálculo 11 (mensal), 2 -&gt; cálculo 32 (13º).  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Anterior diz "Sim".</t>
         </is>
       </c>
     </row>
@@ -48151,12 +48151,12 @@
       <c r="P29" s="38" t="n"/>
       <c r="Q29" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R29" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S29" s="41" t="n">
@@ -48237,7 +48237,7 @@
       </c>
       <c r="R30" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S30" s="41" t="n">
@@ -48434,7 +48434,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -48513,7 +48513,7 @@
       </c>
       <c r="M16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N16" s="30" t="inlineStr">
@@ -50310,7 +50310,7 @@
       </c>
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -50375,7 +50375,7 @@
       </c>
       <c r="L19" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M19" s="30" t="inlineStr">
@@ -51444,7 +51444,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -51509,7 +51509,7 @@
       </c>
       <c r="L15" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M15" s="30" t="inlineStr">
@@ -52147,7 +52147,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -52212,7 +52212,7 @@
       </c>
       <c r="L15" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M15" s="30" t="inlineStr">
@@ -52746,7 +52746,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -52811,7 +52811,7 @@
       </c>
       <c r="L16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M16" s="30" t="inlineStr">
@@ -53698,7 +53698,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -53763,7 +53763,7 @@
       </c>
       <c r="L15" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M15" s="30" t="inlineStr">
@@ -54658,7 +54658,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -54745,7 +54745,7 @@
       </c>
       <c r="M16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N16" s="30" t="inlineStr">
@@ -57040,7 +57040,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fronter_Leiautes 1054 e 1055.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Fronter_Leiautes 1054 e 1055.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -57117,7 +57117,7 @@
       </c>
       <c r="L17" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M17" s="30" t="inlineStr">
@@ -57221,12 +57221,12 @@
       <c r="O18" s="38" t="n"/>
       <c r="P18" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="Q18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R18" s="41" t="n">
@@ -57311,12 +57311,12 @@
       <c r="O19" s="38" t="n"/>
       <c r="P19" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="Q19" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R19" s="41" t="n">
@@ -57398,7 +57398,7 @@
       </c>
       <c r="Q20" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R20" s="41" t="n">
@@ -57473,12 +57473,12 @@
       <c r="O21" s="38" t="n"/>
       <c r="P21" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="Q21" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R21" s="41" t="n">
@@ -57561,12 +57561,12 @@
       <c r="O22" s="38" t="n"/>
       <c r="P22" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="Q22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R22" s="41" t="n">
@@ -57645,12 +57645,12 @@
       <c r="O23" s="38" t="n"/>
       <c r="P23" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="Q23" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R23" s="41" t="n">
@@ -57743,7 +57743,7 @@
       </c>
       <c r="T24" s="38" t="inlineStr">
         <is>
-          <t>CORREÇÃO: o bloco vinculo/sucessaoVinc NÃO aparece em nenhum dos 592 S-2200 analisados. O Fonter mapeou tpInsc genérico, o que traria o tipo de inscrição do PRÓPRIO empregador - dado errado. SUGESTÃO: deixar vazio nesta base.</t>
+          <t>CORREÇÃO: o bloco vinculo/sucessaoVinc NÃO aparece em nenhum dos 592 S-2200 analisados. O Anterior mapeou tpInsc genérico, o que traria o tipo de inscrição do PRÓPRIO empregador - dado errado. SUGESTÃO: deixar vazio nesta base.</t>
         </is>
       </c>
     </row>
@@ -58035,12 +58035,12 @@
       </c>
       <c r="P28" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="Q28" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R28" s="47" t="n"/>
@@ -58113,12 +58113,12 @@
       </c>
       <c r="P29" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="Q29" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R29" s="41" t="n">
@@ -58198,7 +58198,7 @@
       </c>
       <c r="Q30" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R30" s="47" t="n"/>
@@ -58276,7 +58276,7 @@
       </c>
       <c r="Q31" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="R31" s="47" t="n"/>
@@ -58468,7 +58468,7 @@
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fronter_Leiautes 1054 e 1055.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Fronter_Leiautes 1054 e 1055.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -58538,7 +58538,7 @@
       </c>
       <c r="M17" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N17" s="30" t="inlineStr">
@@ -58643,12 +58643,12 @@
       <c r="P18" s="38" t="n"/>
       <c r="Q18" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R18" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S18" s="41" t="n">
@@ -58736,12 +58736,12 @@
       <c r="P19" s="38" t="n"/>
       <c r="Q19" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R19" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S19" s="41" t="n">
@@ -58824,7 +58824,7 @@
       </c>
       <c r="R20" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S20" s="41" t="n">
@@ -58904,12 +58904,12 @@
       </c>
       <c r="Q21" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R21" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="S21" s="41" t="n">
@@ -58993,12 +58993,12 @@
       <c r="P22" s="38" t="n"/>
       <c r="Q22" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R22" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S22" s="49" t="n">
@@ -59082,12 +59082,12 @@
       <c r="P23" s="38" t="n"/>
       <c r="Q23" s="38" t="inlineStr">
         <is>
-          <t>conforme Fonter</t>
+          <t>conforme Anterior</t>
         </is>
       </c>
       <c r="R23" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S23" s="49" t="n">
@@ -59159,12 +59159,12 @@
       <c r="P24" s="38" t="n"/>
       <c r="Q24" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R24" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S24" s="49" t="n">
@@ -59236,12 +59236,12 @@
       <c r="P25" s="38" t="n"/>
       <c r="Q25" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R25" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S25" s="49" t="n">
@@ -59321,12 +59321,12 @@
       </c>
       <c r="Q26" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R26" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S26" s="60" t="n">
@@ -59339,7 +59339,7 @@
       </c>
       <c r="U26" s="38" t="inlineStr">
         <is>
-          <t>CORREÇÃO: a tag é infoEstagiario/vlrBolsa (16,4% dos S-2300). O Fonter escreveu 'remuneracao' e eu sugeri remuneracao/vrSalFx, que existe em apenas 0,5%. SUGESTÃO: vlrBolsa como fonte primária.</t>
+          <t>CORREÇÃO: a tag é infoEstagiario/vlrBolsa (16,4% dos S-2300). O Anterior escreveu 'remuneracao' e eu sugeri remuneracao/vrSalFx, que existe em apenas 0,5%. SUGESTÃO: vlrBolsa como fonte primária.</t>
         </is>
       </c>
     </row>
@@ -59402,12 +59402,12 @@
       <c r="P27" s="38" t="n"/>
       <c r="Q27" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R27" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S27" s="49" t="n">
@@ -59488,7 +59488,7 @@
       </c>
       <c r="R28" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S28" s="49" t="n">
@@ -59573,7 +59573,7 @@
       </c>
       <c r="R29" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="S29" s="49" t="n">
@@ -59645,12 +59645,12 @@
       </c>
       <c r="Q30" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R30" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S30" s="47" t="n"/>
@@ -59729,7 +59729,7 @@
       </c>
       <c r="R31" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S31" s="47" t="n"/>
@@ -59800,7 +59800,7 @@
       </c>
       <c r="R32" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S32" s="47" t="n"/>
@@ -59878,7 +59878,7 @@
       </c>
       <c r="Q33" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R33" s="40" t="inlineStr">
@@ -59959,12 +59959,12 @@
       <c r="P34" s="38" t="n"/>
       <c r="Q34" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="R34" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="S34" s="49" t="n">
@@ -67584,7 +67584,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -67654,7 +67654,7 @@
       </c>
       <c r="M16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="N16" s="30" t="inlineStr">
@@ -77293,13 +77293,13 @@
     <row r="3">
       <c r="A3" s="69" t="inlineStr">
         <is>
-          <t>Mapeamento Fonter</t>
+          <t>Mapeamento Anterior</t>
         </is>
       </c>
       <c r="B3" s="71" t="n"/>
       <c r="C3" s="69" t="inlineStr">
         <is>
-          <t>Colunas dos eventos (S-2200, S-2205, ...) e Observações. Vem das planilhas Fonter, sem alteração.</t>
+          <t>Colunas dos eventos (S-2200, S-2205, ...) e Observações. Vem das planilhas Anterior, sem alteração.</t>
         </is>
       </c>
     </row>
@@ -77350,7 +77350,7 @@
     <row r="8">
       <c r="A8" s="74" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="B8" s="69" t="n"/>
@@ -77363,26 +77363,26 @@
     <row r="9">
       <c r="A9" s="75" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="B9" s="69" t="n"/>
       <c r="C9" s="69" t="inlineStr">
         <is>
-          <t>Base do Fonter mantida; a revisão só qualificou o caminho completo ou acrescentou a regra de transformação.</t>
+          <t>Base do Anterior mantida; a revisão só qualificou o caminho completo ou acrescentou a regra de transformação.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28.8" customHeight="1" s="104">
       <c r="A10" s="76" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="B10" s="69" t="n"/>
       <c r="C10" s="69" t="inlineStr">
         <is>
-          <t>A revisão SUBSTITUIU o mapeamento Fonter - tag inexistente, evento errado ou origem melhor. É aqui que vocês devem olhar primeiro.</t>
+          <t>A revisão SUBSTITUIU o mapeamento Anterior - tag inexistente, evento errado ou origem melhor. É aqui que vocês devem olhar primeiro.</t>
         </is>
       </c>
     </row>
@@ -77395,7 +77395,7 @@
       <c r="B11" s="69" t="n"/>
       <c r="C11" s="69" t="inlineStr">
         <is>
-          <t>Leiaute ou campo que o Fonter não mapeava; definição proposta a partir dos XMLs.</t>
+          <t>Leiaute ou campo que o Anterior não mapeava; definição proposta a partir dos XMLs.</t>
         </is>
       </c>
     </row>
@@ -77439,7 +77439,7 @@
       <c r="B15" s="69" t="n"/>
       <c r="C15" s="69" t="inlineStr">
         <is>
-          <t>Fonter bate com o XML. A coluna Sugestão fica vazia.</t>
+          <t>Anterior bate com o XML. A coluna Sugestão fica vazia.</t>
         </is>
       </c>
     </row>
@@ -77465,7 +77465,7 @@
       <c r="B17" s="69" t="n"/>
       <c r="C17" s="69" t="inlineStr">
         <is>
-          <t>Fonter e a análise dos XMLs apontam origens diferentes - DECIDIR.</t>
+          <t>Anterior e a análise dos XMLs apontam origens diferentes - DECIDIR.</t>
         </is>
       </c>
     </row>
@@ -77491,7 +77491,7 @@
       <c r="B19" s="69" t="n"/>
       <c r="C19" s="69" t="inlineStr">
         <is>
-          <t>Fonter manda vazio ou Fonte: Relatórios, mas o dado está no XML.</t>
+          <t>Anterior manda vazio ou Fonte: Relatórios, mas o dado está no XML.</t>
         </is>
       </c>
     </row>
@@ -77504,7 +77504,7 @@
       <c r="B20" s="69" t="n"/>
       <c r="C20" s="69" t="inlineStr">
         <is>
-          <t>Leiaute sem mapeamento Fonter; origem proposta a partir dos XMLs.</t>
+          <t>Leiaute sem mapeamento Anterior; origem proposta a partir dos XMLs.</t>
         </is>
       </c>
     </row>
@@ -77657,7 +77657,7 @@
       <c r="B33" s="69" t="n"/>
       <c r="C33" s="69" t="inlineStr">
         <is>
-          <t>Cores mantidas do padrão Fonter</t>
+          <t>Cores mantidas do padrão Anterior</t>
         </is>
       </c>
     </row>
@@ -77753,7 +77753,7 @@
       <c r="B41" s="69" t="n"/>
       <c r="C41" s="69" t="inlineStr">
         <is>
-          <t>Os 30 campos onde a obrigatoriedade do leiaute oficial v2.1 diverge da planilha Fonter. O detalhe está na coluna Sugestão.</t>
+          <t>Os 30 campos onde a obrigatoriedade do leiaute oficial v2.1 diverge da planilha Anterior. O detalhe está na coluna Sugestão.</t>
         </is>
       </c>
     </row>
@@ -77766,7 +77766,7 @@
       <c r="B42" s="69" t="n"/>
       <c r="C42" s="69" t="inlineStr">
         <is>
-          <t>Verde = tinha mapeamento Fonter | Âmbar = proposta nova | Cinza = sem origem no eSocial.</t>
+          <t>Verde = tinha mapeamento Anterior | Âmbar = proposta nova | Cinza = sem origem no eSocial.</t>
         </is>
       </c>
     </row>
@@ -77786,7 +77786,7 @@
   • declarado — o campo já tem caminho do evento na coluna Caminho no XML;
   • equivalente — o mesmo caminho relativo existe dentro do evento TSVE.
 Tag que apenas coincide de nome, em outro bloco, NÃO foi preenchida.
-Ficam junto das demais colunas por evento, pintadas de roxo como tudo que este projeto acrescentou; as verdes são do mapeamento Fonter original.</t>
+Ficam junto das demais colunas por evento, pintadas de roxo como tudo que este projeto acrescentou; as verdes são do mapeamento Anterior original.</t>
         </is>
       </c>
     </row>
@@ -77913,7 +77913,7 @@
       </c>
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -77995,7 +77995,7 @@
       </c>
       <c r="L15" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M15" s="30" t="inlineStr">
@@ -79331,7 +79331,7 @@
       </c>
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>Fonter (Fonter_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
+          <t>Anterior (Anterior_Leiautes HCM_v5_20250729.xlsx) + revisão sobre os XMLs</t>
         </is>
       </c>
     </row>
@@ -79433,7 +79433,7 @@
       </c>
       <c r="P16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="Q16" s="30" t="inlineStr">
@@ -79541,12 +79541,12 @@
       </c>
       <c r="T17" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="U17" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="V17" s="47" t="n"/>
@@ -79739,12 +79739,12 @@
       <c r="S19" s="38" t="n"/>
       <c r="T19" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="U19" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="V19" s="55" t="n">
@@ -79839,12 +79839,12 @@
       <c r="S20" s="38" t="n"/>
       <c r="T20" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="U20" s="54" t="inlineStr">
         <is>
-          <t>Fonter (ajustado)</t>
+          <t>Anterior (ajustado)</t>
         </is>
       </c>
       <c r="V20" s="55" t="n">
@@ -79857,7 +79857,7 @@
       </c>
       <c r="X20" s="38" t="inlineStr">
         <is>
-          <t>Coincide (nmCargo). SUGESTÃO: preferir S-1030 dadosCargo/nmCargo.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Fonter diz "Sim". V12: acrescentado o bloco cargoFuncao do trabalhador sem vinculo. Sem isso a linha vinda de um S-2300 caia na busca por nome de tag e virava pendencia. Presenca na amostra: S-2300 24,9%, S-2306 4,9%.</t>
+          <t>Coincide (nmCargo). SUGESTÃO: preferir S-1030 dadosCargo/nmCargo.  |  OBRIGATORIEDADE: leiaute oficial v2.1 diz "Não", Anterior diz "Sim". V12: acrescentado o bloco cargoFuncao do trabalhador sem vinculo. Sem isso a linha vinda de um S-2300 caia na busca por nome de tag e virava pendencia. Presenca na amostra: S-2300 24,9%, S-2306 4,9%.</t>
         </is>
       </c>
     </row>
@@ -79943,12 +79943,12 @@
       </c>
       <c r="T21" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="U21" s="57" t="inlineStr">
         <is>
-          <t>Revisão (substitui Fonter)</t>
+          <t>Revisão (substitui Anterior)</t>
         </is>
       </c>
       <c r="V21" s="41" t="n">
@@ -79961,7 +79961,7 @@
       </c>
       <c r="X21" s="38" t="inlineStr">
         <is>
-          <t>CORREÇÃO: a tag CBOCargo do Fonter EXISTE - achei em 4,1% dos S-2200 e 68,8% dos S-2206 (bloco infoContrato inline, usado quando o empregador não usa tabela de cargos). Eu havia classificado como erro de tag; estava errado. Mesmo assim o S-1030 cobre 100% dos cargos com codCBO. SUGESTÃO: fonte primária S-1030 dadosCargo/codCBO, e CBOCargo como fallback. V12: acrescentado o CBO do proprio evento de admissao como alternativa. A fonte principal continua o S-1030; a alternativa cobre o cliente que nao envia a tabela de cargos. Presenca medida na amostra: 4,1% dos 19.526 S-2200, 25,2% dos 1.117 S-2300 e 4,9% dos 223 S-2306 da massa de teste completa. E de onde o Ponto P le.</t>
+          <t>CORREÇÃO: a tag CBOCargo do Anterior EXISTE - achei em 4,1% dos S-2200 e 68,8% dos S-2206 (bloco infoContrato inline, usado quando o empregador não usa tabela de cargos). Eu havia classificado como erro de tag; estava errado. Mesmo assim o S-1030 cobre 100% dos cargos com codCBO. SUGESTÃO: fonte primária S-1030 dadosCargo/codCBO, e CBOCargo como fallback. V12: acrescentado o CBO do proprio evento de admissao como alternativa. A fonte principal continua o S-1030; a alternativa cobre o cliente que nao envia a tabela de cargos. Presenca medida na amostra: 4,1% dos 19.526 S-2200, 25,2% dos 1.117 S-2300 e 4,9% dos 223 S-2306 da massa de teste completa. E de onde o Ponto P le.</t>
         </is>
       </c>
     </row>
@@ -80029,7 +80029,7 @@
       <c r="S22" s="38" t="n"/>
       <c r="T22" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="U22" s="40" t="inlineStr">
@@ -80111,12 +80111,12 @@
       </c>
       <c r="T23" s="43" t="inlineStr">
         <is>
-          <t>sem De/Para (conforme Fonter)</t>
+          <t>sem De/Para (conforme Anterior)</t>
         </is>
       </c>
       <c r="U23" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="V23" s="55" t="n">
@@ -80202,7 +80202,7 @@
       </c>
       <c r="U24" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="V24" s="47" t="n"/>
@@ -80282,7 +80282,7 @@
       </c>
       <c r="U25" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="V25" s="47" t="n"/>
@@ -80354,7 +80354,7 @@
       </c>
       <c r="U26" s="51" t="inlineStr">
         <is>
-          <t>Fonter</t>
+          <t>Anterior</t>
         </is>
       </c>
       <c r="V26" s="47" t="n"/>
@@ -80537,7 +80537,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Fonter anterior</t>
+          <t>Proposto a partir dos XMLs do eSocial - sem mapeamento Anterior anterior</t>
         </is>
       </c>
     </row>
@@ -80602,7 +80602,7 @@
       </c>
       <c r="L16" s="29" t="inlineStr">
         <is>
-          <t>Observações (Fonter)</t>
+          <t>Observações (Anterior)</t>
         </is>
       </c>
       <c r="M16" s="30" t="inlineStr">

</xml_diff>